<commit_message>
missing some shot charts
</commit_message>
<xml_diff>
--- a/ShotCharts/shot_zones_2025_26.xlsx
+++ b/ShotCharts/shot_zones_2025_26.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="526">
   <si>
     <t>Player</t>
   </si>
@@ -1577,6 +1577,21 @@
   </si>
   <si>
     <t>Trey Jemison</t>
+  </si>
+  <si>
+    <t>A.J. Green</t>
+  </si>
+  <si>
+    <t>Nicolas Claxton</t>
+  </si>
+  <si>
+    <t>Alexandre Sarr</t>
+  </si>
+  <si>
+    <t>AJ Lawson</t>
+  </si>
+  <si>
+    <t>Carlton Carrington</t>
   </si>
 </sst>
 </file>
@@ -1934,7 +1949,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V500"/>
+  <dimension ref="A1:V505"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -35937,6 +35952,346 @@
         <v>0</v>
       </c>
     </row>
+    <row r="501" spans="1:22">
+      <c r="A501" t="s">
+        <v>521</v>
+      </c>
+      <c r="B501">
+        <v>417</v>
+      </c>
+      <c r="C501">
+        <v>0.0312</v>
+      </c>
+      <c r="D501">
+        <v>13</v>
+      </c>
+      <c r="E501">
+        <v>8</v>
+      </c>
+      <c r="F501">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="G501">
+        <v>0.0312</v>
+      </c>
+      <c r="H501">
+        <v>13</v>
+      </c>
+      <c r="I501">
+        <v>8</v>
+      </c>
+      <c r="J501">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="K501">
+        <v>0.0408</v>
+      </c>
+      <c r="L501">
+        <v>17</v>
+      </c>
+      <c r="M501">
+        <v>5</v>
+      </c>
+      <c r="N501">
+        <v>0.2941</v>
+      </c>
+      <c r="O501">
+        <v>0.271</v>
+      </c>
+      <c r="P501">
+        <v>113</v>
+      </c>
+      <c r="Q501">
+        <v>58</v>
+      </c>
+      <c r="R501">
+        <v>0.5133</v>
+      </c>
+      <c r="S501">
+        <v>0.6259</v>
+      </c>
+      <c r="T501">
+        <v>261</v>
+      </c>
+      <c r="U501">
+        <v>101</v>
+      </c>
+      <c r="V501">
+        <v>0.387</v>
+      </c>
+    </row>
+    <row r="502" spans="1:22">
+      <c r="A502" t="s">
+        <v>522</v>
+      </c>
+      <c r="B502">
+        <v>463</v>
+      </c>
+      <c r="C502">
+        <v>0.6069</v>
+      </c>
+      <c r="D502">
+        <v>281</v>
+      </c>
+      <c r="E502">
+        <v>199</v>
+      </c>
+      <c r="F502">
+        <v>0.7082000000000001</v>
+      </c>
+      <c r="G502">
+        <v>0.3089</v>
+      </c>
+      <c r="H502">
+        <v>143</v>
+      </c>
+      <c r="I502">
+        <v>60</v>
+      </c>
+      <c r="J502">
+        <v>0.4196</v>
+      </c>
+      <c r="K502">
+        <v>0.0497</v>
+      </c>
+      <c r="L502">
+        <v>23</v>
+      </c>
+      <c r="M502">
+        <v>12</v>
+      </c>
+      <c r="N502">
+        <v>0.5217000000000001</v>
+      </c>
+      <c r="O502">
+        <v>0.0022</v>
+      </c>
+      <c r="P502">
+        <v>1</v>
+      </c>
+      <c r="Q502">
+        <v>0</v>
+      </c>
+      <c r="R502">
+        <v>0</v>
+      </c>
+      <c r="S502">
+        <v>0.0324</v>
+      </c>
+      <c r="T502">
+        <v>15</v>
+      </c>
+      <c r="U502">
+        <v>3</v>
+      </c>
+      <c r="V502">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="503" spans="1:22">
+      <c r="A503" t="s">
+        <v>523</v>
+      </c>
+      <c r="B503">
+        <v>575</v>
+      </c>
+      <c r="C503">
+        <v>0.3652</v>
+      </c>
+      <c r="D503">
+        <v>210</v>
+      </c>
+      <c r="E503">
+        <v>151</v>
+      </c>
+      <c r="F503">
+        <v>0.719</v>
+      </c>
+      <c r="G503">
+        <v>0.3322</v>
+      </c>
+      <c r="H503">
+        <v>191</v>
+      </c>
+      <c r="I503">
+        <v>76</v>
+      </c>
+      <c r="J503">
+        <v>0.3979</v>
+      </c>
+      <c r="K503">
+        <v>0.09569999999999999</v>
+      </c>
+      <c r="L503">
+        <v>55</v>
+      </c>
+      <c r="M503">
+        <v>18</v>
+      </c>
+      <c r="N503">
+        <v>0.3273</v>
+      </c>
+      <c r="O503">
+        <v>0.0157</v>
+      </c>
+      <c r="P503">
+        <v>9</v>
+      </c>
+      <c r="Q503">
+        <v>3</v>
+      </c>
+      <c r="R503">
+        <v>0.3333</v>
+      </c>
+      <c r="S503">
+        <v>0.1913</v>
+      </c>
+      <c r="T503">
+        <v>110</v>
+      </c>
+      <c r="U503">
+        <v>37</v>
+      </c>
+      <c r="V503">
+        <v>0.3364</v>
+      </c>
+    </row>
+    <row r="504" spans="1:22">
+      <c r="A504" t="s">
+        <v>524</v>
+      </c>
+      <c r="B504">
+        <v>41</v>
+      </c>
+      <c r="C504">
+        <v>0.3415</v>
+      </c>
+      <c r="D504">
+        <v>14</v>
+      </c>
+      <c r="E504">
+        <v>7</v>
+      </c>
+      <c r="F504">
+        <v>0.5</v>
+      </c>
+      <c r="G504">
+        <v>0.122</v>
+      </c>
+      <c r="H504">
+        <v>5</v>
+      </c>
+      <c r="I504">
+        <v>1</v>
+      </c>
+      <c r="J504">
+        <v>0.2</v>
+      </c>
+      <c r="K504">
+        <v>0</v>
+      </c>
+      <c r="L504">
+        <v>0</v>
+      </c>
+      <c r="M504">
+        <v>0</v>
+      </c>
+      <c r="N504">
+        <v>0</v>
+      </c>
+      <c r="O504">
+        <v>0.3659</v>
+      </c>
+      <c r="P504">
+        <v>15</v>
+      </c>
+      <c r="Q504">
+        <v>5</v>
+      </c>
+      <c r="R504">
+        <v>0.3333</v>
+      </c>
+      <c r="S504">
+        <v>0.1707</v>
+      </c>
+      <c r="T504">
+        <v>7</v>
+      </c>
+      <c r="U504">
+        <v>3</v>
+      </c>
+      <c r="V504">
+        <v>0.4286</v>
+      </c>
+    </row>
+    <row r="505" spans="1:22">
+      <c r="A505" t="s">
+        <v>525</v>
+      </c>
+      <c r="B505">
+        <v>507</v>
+      </c>
+      <c r="C505">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="D505">
+        <v>36</v>
+      </c>
+      <c r="E505">
+        <v>16</v>
+      </c>
+      <c r="F505">
+        <v>0.4444</v>
+      </c>
+      <c r="G505">
+        <v>0.1321</v>
+      </c>
+      <c r="H505">
+        <v>67</v>
+      </c>
+      <c r="I505">
+        <v>23</v>
+      </c>
+      <c r="J505">
+        <v>0.3433</v>
+      </c>
+      <c r="K505">
+        <v>0.2012</v>
+      </c>
+      <c r="L505">
+        <v>102</v>
+      </c>
+      <c r="M505">
+        <v>45</v>
+      </c>
+      <c r="N505">
+        <v>0.4412</v>
+      </c>
+      <c r="O505">
+        <v>0.0769</v>
+      </c>
+      <c r="P505">
+        <v>39</v>
+      </c>
+      <c r="Q505">
+        <v>14</v>
+      </c>
+      <c r="R505">
+        <v>0.359</v>
+      </c>
+      <c r="S505">
+        <v>0.5187</v>
+      </c>
+      <c r="T505">
+        <v>263</v>
+      </c>
+      <c r="U505">
+        <v>101</v>
+      </c>
+      <c r="V505">
+        <v>0.384</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>